<commit_message>
feat(s22): S22-P5c pack — importer blockers (business unit / location), prototype v5, synthetic fixture with Zeta Unlisted; scoreboard rows P5c-1…4
Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/api/tests/forecast/fixtures/forecast_model_synthetic.xlsx
+++ b/api/tests/forecast/fixtures/forecast_model_synthetic.xlsx
@@ -12,7 +12,8 @@
     <sheet name="Alpha" sheetId="3" state="visible" r:id="rId3"/>
     <sheet name="Beta" sheetId="4" state="visible" r:id="rId4"/>
     <sheet name="Gamma Health-VMS" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet name="Delta Closed" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet name="Zeta Unlisted" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet name="Delta Closed" sheetId="7" state="visible" r:id="rId7"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -421,7 +422,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="B5:E15"/>
+  <dimension ref="B5:E23"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="5">
@@ -588,6 +589,56 @@
       <c r="E15" t="inlineStr">
         <is>
           <t>T&amp;M</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>Subtotal</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>Total</t>
+        </is>
+      </c>
+    </row>
+    <row r="18"/>
+    <row r="19">
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>Client</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>ST21</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>ITA</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>RR</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>Total</t>
         </is>
       </c>
     </row>
@@ -2122,6 +2173,203 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
+  <dimension ref="A1:M7"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="I1" t="n">
+        <v>2026</v>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>ZETA</t>
+        </is>
+      </c>
+      <c r="I2" t="inlineStr">
+        <is>
+          <t>Actual</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="I3" t="inlineStr">
+        <is>
+          <t>January</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>Resource</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>Role</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>Team/SOW</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>Type</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>SOW Start Date</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>SOW End Date</t>
+        </is>
+      </c>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>Location</t>
+        </is>
+      </c>
+      <c r="H4" t="inlineStr">
+        <is>
+          <t>Rate</t>
+        </is>
+      </c>
+      <c r="I4" t="inlineStr">
+        <is>
+          <t>Max Days</t>
+        </is>
+      </c>
+      <c r="J4" t="inlineStr">
+        <is>
+          <t>Vacation Days</t>
+        </is>
+      </c>
+      <c r="K4" t="inlineStr">
+        <is>
+          <t>Unplanned Leave</t>
+        </is>
+      </c>
+      <c r="L4" t="inlineStr">
+        <is>
+          <t>Max Billing</t>
+        </is>
+      </c>
+      <c r="M4" t="inlineStr">
+        <is>
+          <t>Billing</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>Person Z1</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>Engineer</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>SOW #4</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>Managed Services</t>
+        </is>
+      </c>
+      <c r="E5" s="1" t="n">
+        <v>46023</v>
+      </c>
+      <c r="F5" s="1" t="n">
+        <v>46203</v>
+      </c>
+      <c r="H5" t="n">
+        <v>60</v>
+      </c>
+      <c r="I5" t="n">
+        <v>20</v>
+      </c>
+      <c r="L5" t="n">
+        <v>9600</v>
+      </c>
+      <c r="M5" t="n">
+        <v>9600</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>Person Z2</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>Engineer</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>SOW #4</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>Managed Services</t>
+        </is>
+      </c>
+      <c r="E6" s="1" t="n">
+        <v>46023</v>
+      </c>
+      <c r="F6" s="1" t="n">
+        <v>46203</v>
+      </c>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>US</t>
+        </is>
+      </c>
+      <c r="H6" t="n">
+        <v>60</v>
+      </c>
+      <c r="I6" t="n">
+        <v>20</v>
+      </c>
+      <c r="L6" t="n">
+        <v>9600</v>
+      </c>
+      <c r="M6" t="n">
+        <v>9600</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>Total</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
   <dimension ref="A1:M6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>

</xml_diff>

<commit_message>
feat(s22): S22-P5 final pack — importer re-audited (row_key identity, actual hours from the invoice, extension day-after, assumptions section, streaming read), contract import_key; fixtures regenerated; scoreboard rows P5f-1…5
45 forecast tests pass first.

Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/api/tests/forecast/fixtures/forecast_model_synthetic.xlsx
+++ b/api/tests/forecast/fixtures/forecast_model_synthetic.xlsx
@@ -1750,7 +1750,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A2:AE8"/>
+  <dimension ref="A2:AE10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="2">
@@ -2157,6 +2157,169 @@
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
+        <is>
+          <t>Person G3</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>Analyst</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>VMS</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>Staffing</t>
+        </is>
+      </c>
+      <c r="E8" s="1" t="n">
+        <v>45992</v>
+      </c>
+      <c r="F8" s="1" t="n">
+        <v>46112</v>
+      </c>
+      <c r="H8" s="1" t="n">
+        <v>46203</v>
+      </c>
+      <c r="I8" t="inlineStr">
+        <is>
+          <t>US</t>
+        </is>
+      </c>
+      <c r="J8" t="n">
+        <v>90</v>
+      </c>
+      <c r="K8" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="L8" t="n">
+        <v>168</v>
+      </c>
+      <c r="M8" t="n">
+        <v>160</v>
+      </c>
+      <c r="O8" t="n">
+        <v>15120</v>
+      </c>
+      <c r="P8" t="n">
+        <v>14400</v>
+      </c>
+      <c r="Q8" t="n">
+        <v>160</v>
+      </c>
+      <c r="R8" t="n">
+        <v>152</v>
+      </c>
+      <c r="T8" t="n">
+        <v>14400</v>
+      </c>
+      <c r="U8" t="n">
+        <v>13680</v>
+      </c>
+      <c r="V8" t="n">
+        <v>176</v>
+      </c>
+      <c r="Y8" t="n">
+        <v>15840</v>
+      </c>
+      <c r="AA8" t="n">
+        <v>176</v>
+      </c>
+      <c r="AD8" t="n">
+        <v>15840</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>Person G4</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>Analyst</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>VMS</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>Staffing</t>
+        </is>
+      </c>
+      <c r="E9" s="1" t="n">
+        <v>45992</v>
+      </c>
+      <c r="F9" s="1" t="n">
+        <v>46112</v>
+      </c>
+      <c r="G9" s="1" t="n">
+        <v>46112</v>
+      </c>
+      <c r="H9" s="1" t="n">
+        <v>46295</v>
+      </c>
+      <c r="I9" t="inlineStr">
+        <is>
+          <t>US</t>
+        </is>
+      </c>
+      <c r="J9" t="n">
+        <v>90</v>
+      </c>
+      <c r="K9" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="L9" t="n">
+        <v>168</v>
+      </c>
+      <c r="M9" t="n">
+        <v>160</v>
+      </c>
+      <c r="O9" t="n">
+        <v>15120</v>
+      </c>
+      <c r="P9" t="n">
+        <v>14400</v>
+      </c>
+      <c r="Q9" t="n">
+        <v>160</v>
+      </c>
+      <c r="R9" t="n">
+        <v>152</v>
+      </c>
+      <c r="T9" t="n">
+        <v>14400</v>
+      </c>
+      <c r="U9" t="n">
+        <v>13680</v>
+      </c>
+      <c r="V9" t="n">
+        <v>176</v>
+      </c>
+      <c r="Y9" t="n">
+        <v>15840</v>
+      </c>
+      <c r="AA9" t="n">
+        <v>176</v>
+      </c>
+      <c r="AD9" t="n">
+        <v>15840</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
         <is>
           <t>Total</t>
         </is>
@@ -2173,7 +2336,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M7"/>
+  <dimension ref="A1:M9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -2354,6 +2517,99 @@
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
+        <is>
+          <t>TBC</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>Engineer</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>SOW #4</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>Managed Services</t>
+        </is>
+      </c>
+      <c r="E7" s="1" t="n">
+        <v>46023</v>
+      </c>
+      <c r="F7" s="1" t="n">
+        <v>46203</v>
+      </c>
+      <c r="G7" t="inlineStr">
+        <is>
+          <t>US</t>
+        </is>
+      </c>
+      <c r="H7" t="n">
+        <v>60</v>
+      </c>
+      <c r="I7" t="n">
+        <v>20</v>
+      </c>
+      <c r="J7" t="n">
+        <v>1</v>
+      </c>
+      <c r="L7" t="n">
+        <v>9600</v>
+      </c>
+      <c r="M7" t="n">
+        <v>8400</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>TBC</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>Engineer</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>SOW #4</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>Managed Services</t>
+        </is>
+      </c>
+      <c r="E8" s="1" t="n">
+        <v>46023</v>
+      </c>
+      <c r="F8" s="1" t="n">
+        <v>46203</v>
+      </c>
+      <c r="G8" t="inlineStr">
+        <is>
+          <t>US</t>
+        </is>
+      </c>
+      <c r="H8" t="n">
+        <v>60</v>
+      </c>
+      <c r="I8" t="n">
+        <v>20</v>
+      </c>
+      <c r="L8" t="n">
+        <v>9600</v>
+      </c>
+      <c r="M8" t="n">
+        <v>9600</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
         <is>
           <t>Total</t>
         </is>

</xml_diff>